<commit_message>
ledger: add tonight's three works, and rebuild the spreadsheet
tools/register.artifact.html gains SOPPO / MUSUBI / SHIMA at the head of
WORKS (55 entries, matching works.csv exactly), and oto-2-works.xlsx is
regenerated from works.csv. The owner's hand-written 〇/△ and memo columns
were carried across for all 49 works that already had them.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LjZQcfFrqobmdEwsM7AJ5C
</commit_message>
<xml_diff>
--- a/oto-2-works.xlsx
+++ b/oto-2-works.xlsx
@@ -13,9 +13,9 @@
     <sheet name="使い方" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ゲーム'!$A$1:$G$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'楽器'!$A$1:$G$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'エフェクト'!$A$1:$G$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1016,10 +1016,72 @@
         </is>
       </c>
     </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>UGUISU</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>梅の枝の鶯と鳴き交わす五番勝負。鶯の鳴いたふしを声か口笛で返す。見ているのは高さではなく音と音の隔たりなのでどんな声でもよい。</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>SOPPO</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>紙芝居の舞台で狸と向かい合う五番勝負のあっち向いてホイ。じゃんけんに勝てば指をさす側、負ければ顔をそむける側。ホイの一瞬にさされた向きへ顔を向けたら取られ、どこへも向かなければそれも取られる。</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>ゲーム</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G12"/>
+  <autoFilter ref="A1:G14"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1035,6 +1097,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -1047,7 +1111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1406,10 +1470,72 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>MUKKURI</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>音の高さを変えない口琴。弁は一つの高さで鳴りつづけ変わるのは口のなかの空洞だけ。どの倍音が選ばれているかが口のなかに見える。</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>楽器</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>MUSUBI</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>手が四本まで見える楽器。一本の手は細く濁った声しか出せず、もう一方の手へ近づけるとあいだに組紐が伸びて唸りがほどけて澄む。近づけきると結ばれて金の結び目が残る。ふたりでも編める。</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>楽器</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G11"/>
+  <autoFilter ref="A1:G13"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1424,6 +1550,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -1436,7 +1564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2002,7 +2130,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>カメラ映像を明るさで切り分け色紙を重ねた切り絵にする。手を開くと層が離れて影が落ち動かすと視差でずれる。</t>
+          <t>カメラ映像を明るさで切り分け色紙を重ねた切り絵にする。輪郭は画素ではなく本物の曲線なので拡大しても刃の跡。手を開くと層が離れる。</t>
         </is>
       </c>
       <c r="F18" s="6" t="n"/>
@@ -2353,10 +2481,72 @@
         </is>
       </c>
     </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>SUMINAGASHI</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>水面に墨を落として櫛で梳く本物の墨流し。拡散が一度も起きないので何十回梳いても墨は濁らず細い筋になって伸びる。</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n"/>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>〇</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>SHIMA</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>細い罫を二枚かさねるとどちらにも無い太い縞が出る。二枚目はカメラの明るさで撓むので縞はあなたの形の等高線になる。角度と間隔がそろうと縞間隔は無限に伸びて消え唸りも止まる。</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>エフェクト</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G29"/>
+  <autoFilter ref="A1:G31"/>
   <dataValidations count="1">
-    <dataValidation sqref="B2:B29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
+    <dataValidation sqref="B2:B31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="〇 / △ / × のどれかを選んでください" prompt="〇=このままでよい / △=後日なおす / ×=作り直す" type="list">
       <formula1>"〇,△,×"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2389,6 +2579,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
@@ -2527,15 +2719,15 @@
         </is>
       </c>
       <c r="B15" s="13">
-        <f>COUNTIF(ゲーム!$B$2:$B$12,"〇")</f>
+        <f>COUNTIF(ゲーム!$B$2:$B$14,"〇")</f>
         <v/>
       </c>
       <c r="C15" s="13">
-        <f>COUNTIF(楽器!$B$2:$B$11,"〇")</f>
+        <f>COUNTIF(楽器!$B$2:$B$13,"〇")</f>
         <v/>
       </c>
       <c r="D15" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$29,"〇")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$31,"〇")</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -2550,15 +2742,15 @@
         </is>
       </c>
       <c r="B16" s="13">
-        <f>COUNTIF(ゲーム!$B$2:$B$12,"△")</f>
+        <f>COUNTIF(ゲーム!$B$2:$B$14,"△")</f>
         <v/>
       </c>
       <c r="C16" s="13">
-        <f>COUNTIF(楽器!$B$2:$B$11,"△")</f>
+        <f>COUNTIF(楽器!$B$2:$B$13,"△")</f>
         <v/>
       </c>
       <c r="D16" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$29,"△")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$31,"△")</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -2573,15 +2765,15 @@
         </is>
       </c>
       <c r="B17" s="13">
-        <f>COUNTIF(ゲーム!$B$2:$B$12,"×")</f>
+        <f>COUNTIF(ゲーム!$B$2:$B$14,"×")</f>
         <v/>
       </c>
       <c r="C17" s="13">
-        <f>COUNTIF(楽器!$B$2:$B$11,"×")</f>
+        <f>COUNTIF(楽器!$B$2:$B$13,"×")</f>
         <v/>
       </c>
       <c r="D17" s="13">
-        <f>COUNTIF(エフェクト!$B$2:$B$29,"×")</f>
+        <f>COUNTIF(エフェクト!$B$2:$B$31,"×")</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -2596,13 +2788,13 @@
         </is>
       </c>
       <c r="B18" s="15" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C18" s="15" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D18" s="15" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E18" s="16">
         <f>SUM(B18:D18)</f>

</xml_diff>